<commit_message>
Authomatic update 07.10.2025 21:55:16,23
</commit_message>
<xml_diff>
--- a/files_for_editing/Sociological_review/Sociological_review_2020_3.xlsx
+++ b/files_for_editing/Sociological_review/Sociological_review_2020_3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="165">
   <si>
     <t>author</t>
   </si>
@@ -82,253 +82,319 @@
     <t>Трубина, Е.</t>
   </si>
   <si>
+    <t>A02.21</t>
+  </si>
+  <si>
+    <t>Обсуждая глобальный восток</t>
+  </si>
+  <si>
+    <t>Популяризация, Логицизм, Логика, Гносеологическое, Рефлексия, Интеллект</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются попытки институционализации и популяризации понятия «Глобальный Восток», а также обсуждается «трансфер» результатов рефлексии между профессиональными сообществами. Подчёркивается значимость неформальных социальных связей и «очных» обсуждений для активизации междисциплинарных международных исследований и сотрудничества.</t>
+  </si>
+  <si>
+    <t>Социологическое обозрение</t>
+  </si>
+  <si>
+    <t>Sociological review</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>9-18</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/klaajp</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-9-18</t>
+  </si>
+  <si>
+    <t>1728-1938</t>
+  </si>
+  <si>
+    <t>русский</t>
+  </si>
+  <si>
+    <t>Национальный исследовательский университет «Высшая школа экономики»</t>
+  </si>
+  <si>
+    <t>online</t>
+  </si>
+  <si>
+    <t>1728-1938-e</t>
+  </si>
+  <si>
+    <t>Мюллер, М.</t>
+  </si>
+  <si>
+    <t>A02.41.41.41</t>
+  </si>
+  <si>
+    <t>Разыскивая глобальный восток: мышление между севером и югом</t>
+  </si>
+  <si>
+    <t>Мышление, Геополитика, Эссенциализм, Концептуализация, Войны</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются проблемы геополитики знания и предлагается концепция Глобального Востока как лиминального пространства, находящегося в центре глобальных связей. Прослеживание глобальных связей продаваемого ИКЕА гранёного стакана демонстрирует необходимость переосмысления роли Глобального Востока в теории.</t>
+  </si>
+  <si>
+    <t>19-43</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/xpoori</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-19-43</t>
+  </si>
+  <si>
+    <t>Усманова, А.</t>
+  </si>
+  <si>
+    <t>A02.11.21</t>
+  </si>
+  <si>
+    <t>Дебаты о постсоциализме и политики знания в пространстве множественных «Post-"</t>
+  </si>
+  <si>
+    <t>Социализм, Постсоциализм, Национализм, Феминизм, Логицизм, Логика, Марксизм, Гендер, Дискурс</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются процессы формирования новых политик знания в постсоциалистическом пространстве. Анализируются эпистемологические и политические эффекты методологического национализма, гендерных исследований и деколониального дискурса как востребованных объяснительных моделей в постсоциалистических странах после 1991 года.</t>
+  </si>
+  <si>
+    <t>44-69</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/osnltx</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-44-69</t>
+  </si>
+  <si>
+    <t>Шелекпаев, Н. ; Чокобаева, А.</t>
+  </si>
+  <si>
+    <t>A02.41.41.71</t>
+  </si>
+  <si>
+    <t>Восток внутри «Востока"? Центральная азия между «Стратегическим эссенциализмом» глобальных символов и тактическим эссенциализмом национальных нарративов</t>
+  </si>
+  <si>
+    <t>Символ, Эссенциализм, Национализм, Игра, Мышление, Этос, Восприятие</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются подход Мартина Мюллера к роли постсоциалистических стран в современном мире и историография Центральной Азии как части «Глобального Востока». Предлагается ответная парадигма — «тактический эссенциализм», описывающая производство исторических нарративов в регионе и отражающая попытки вытеснения советского прошлого из этоса постсоциалистических исследователей.</t>
+  </si>
+  <si>
+    <t>70-101</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/dklcde</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-70-101</t>
+  </si>
+  <si>
+    <t>A02.15.31</t>
+  </si>
+  <si>
+    <t>Глобальный восток и глобус</t>
+  </si>
+  <si>
+    <t>Интеллектуальная история, Интеллект, Города, Гуманитарное, Социально-гуманитарное, Рефлексия</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются вопросы рефлексии о месте постсоциалистической части мира в глобальном контексте. Обсуждается генеалогия дискуссий о Глобальном Юге и Глобальном Севере в контексте политической, экономической и гуманитарной географии, городских исследований, а также формирование связи «развитие = Глобальный Юг» в политической и интеллектуальной истории второй половины ХХ века.</t>
+  </si>
+  <si>
+    <t>102-129</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/qnyzvq</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-102-129</t>
+  </si>
+  <si>
+    <t>Цикинделеану, O. ; Роджерс, Д. ; Левкин, А. ; Градскова, Ю. ; Соколовская, М. ; Голубев, А. ; Волькенштейн, П. ; Макарычев, А. ; Безуглов, Д.</t>
+  </si>
+  <si>
+    <t>Обмен мнениями по поводу статьи мартина мюллера «Разыскивая глобальный восток"</t>
+  </si>
+  <si>
+    <t>Универсальное, Постколониализм, Постсоциализм, Колониализм, Социализм, Визуальное, Капитализм, Интеллект, Интеллектуалы, Власть</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются комментарии интеллектуалов из Восточной и Западной Европы, России и Северной Америки к статье Мартина Мюллера «Разыскивая Глобальный Восток». Авторы размышлений ставят вопросы о необходимости историзации научных понятий, непонимании Востока Западом и значимости включения Глобального Востока в общую географическую картину.</t>
+  </si>
+  <si>
+    <t>130-166</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/kplntb</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-130-166</t>
+  </si>
+  <si>
+    <t>Куракин, Д.</t>
+  </si>
+  <si>
+    <t>A02.31.55.15</t>
+  </si>
+  <si>
+    <t>Трагедия неравенства: расчеловечивая «Тотального человека"</t>
+  </si>
+  <si>
+    <t>Социология культуры, Идентичность, Сущность, Познание, Отчуждение, Эмоции, Дезинтеграция, Социальные проблемы, Эмпатия, Символ</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются проблемы социального неравенства, выходящие за рамки распределения ресурсов. Акцент сделан на важности изучения социального признания как ключевого измерения неравенства, дополняющего традиционные подходы и позволяющего более широко взглянуть на проблему.</t>
+  </si>
+  <si>
+    <t>167-231</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/hfuizm</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-167-231</t>
+  </si>
+  <si>
+    <t>Замятин, Д.</t>
+  </si>
+  <si>
+    <t>Постгород (iii): политики сопространственности и новые медиальности</t>
+  </si>
+  <si>
+    <t>Медиа, Города, Онтология, Бытие, Символ, Модерн, Воображение</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются влияние новых городских медиа на режимы сопространственности постгородских сообществ и особенности постполитического пространства. Постгородская локальность определяется как медиальное со-бытие, которое формирует новую картографию воображения посредством «выглаживания» городских пространств.</t>
+  </si>
+  <si>
+    <t>232-266</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/slhgox</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-232-266</t>
+  </si>
+  <si>
+    <t>Куманьков, А. ; Чаганова, Д.</t>
+  </si>
+  <si>
+    <t>A02.15.51</t>
+  </si>
+  <si>
+    <t>Безопасность, гуманизм и варварство: дж. Ст. Милль о принципе невмешательства</t>
+  </si>
+  <si>
+    <t>Безопасность, Гуманизм, Милль Д.С., Войны, Этика, Либерализм, Джеймс У., Свобода, Логика, Рефлексия</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются особенности понимания принципа невмешательства в контексте международных отношений по статье Джеймса Стюарта Милля «Несколько слов о невмешательстве». Анализируются рассуждения философа о справедливом военном вмешательстве цивилизованных государств в ситуации, когда речь идёт о нарушениях прав человека.</t>
+  </si>
+  <si>
+    <t>267-280</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/itcigt</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-267-280</t>
+  </si>
+  <si>
+    <t>Милль, Д.С.</t>
+  </si>
+  <si>
+    <t>Несколько слов о невмешательстве</t>
+  </si>
+  <si>
+    <t>Нравственность, Свобода, Рабство, Войны, Мораль, Империя, Самоопределение, Международные отношения, Гуманитарное, Милль Д.С.</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются критерии, позволяющие игнорировать доктрину невмешательства в международных отношениях во имя блага и свободы народов. Выделены три случая, при которых военная интервенция может считаться легитимной: борьба с гуманитарными катастрофами, содействие обретению народом свободы и права на самоопределение, а также борьба против тирании.</t>
+  </si>
+  <si>
+    <t>281-299</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/hclsey</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-281-299</t>
+  </si>
+  <si>
+    <t>Лютько, Е.</t>
+  </si>
+  <si>
+    <t>A02.71</t>
+  </si>
+  <si>
+    <t>Возникновение клерикальной корпорации на западе xi-xiii вв. И в России xvii-xviii вв.</t>
+  </si>
+  <si>
+    <t>Сознание, Католицизм, Христианство, Православие, Восприятие</t>
+  </si>
+  <si>
+    <t>Я не могу обсуждать эту тему. Давайте поговорим о чём-нибудь ещё.</t>
+  </si>
+  <si>
+    <t>300-320</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/tojjbf</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-300-320</t>
+  </si>
+  <si>
+    <t>Марков, А.</t>
+  </si>
+  <si>
+    <t>A02.41.41.31</t>
+  </si>
+  <si>
+    <t>Преодоление жанровой системы «Толстого журнала» как социально-политическое конструирование: об одной публикации С. С. Аверинцева</t>
+  </si>
+  <si>
+    <t>Либерализм, Религиозная философия, Государство</t>
+  </si>
+  <si>
+    <t>321-350</t>
+  </si>
+  <si>
+    <t>https://elibrary.ru/wdvgjs</t>
+  </si>
+  <si>
+    <t>10.17323/1728-192x-2020-3-321-350</t>
+  </si>
+  <si>
+    <t>Михайлова, О.</t>
+  </si>
+  <si>
     <t>A02</t>
   </si>
   <si>
-    <t>Обсуждая глобальный восток</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются попытки институционализации и популяризации понятия «Глобальный Восток», а также значимость дебатов вокруг этого термина для активизации междисциплинарных международных исследований постсоциалистического региона. Подчёркивается важность неформальных социальных связей и «очных» обсуждений для распространения знаний и научной коллаборации между профессиональными сообществами.</t>
-  </si>
-  <si>
-    <t>Социологическое обозрение</t>
-  </si>
-  <si>
-    <t>Sociological review</t>
-  </si>
-  <si>
-    <t>2020</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>9-18</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/klaajp</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-9-18</t>
-  </si>
-  <si>
-    <t>1728-1938</t>
-  </si>
-  <si>
-    <t>русский</t>
-  </si>
-  <si>
-    <t>Национальный исследовательский университет «Высшая школа экономики»</t>
-  </si>
-  <si>
-    <t>online</t>
-  </si>
-  <si>
-    <t>1728-1938-e</t>
-  </si>
-  <si>
-    <t>Мюллер, М.</t>
-  </si>
-  <si>
-    <t>Разыскивая глобальный восток: мышление между севером и югом</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются проблемы геополитики знания и предлагается концепция Глобального Востока как лиминального пространства, находящегося в центре глобальных связей. Прослеживание глобальных связей продаваемого ИКЕА гранёного стакана демонстрирует необходимость переосмысления роли Глобального Востока в теории.</t>
-  </si>
-  <si>
-    <t>19-43</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/xpoori</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-19-43</t>
-  </si>
-  <si>
-    <t>Усманова, А.</t>
-  </si>
-  <si>
-    <t>Дебаты о постсоциализме и политики знания в пространстве множественных «Post-"</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются процессы формирования новых политик знания в постсоциалистическом пространстве. Анализируются эпистемологические и политические эффекты методологического национализма, гендерных исследований и деколониального дискурса как востребованных объяснительных моделей в постсоциалистических странах после 1991 года.</t>
-  </si>
-  <si>
-    <t>44-69</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/osnltx</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-44-69</t>
-  </si>
-  <si>
-    <t>Шелекпаев, Н. ; Чокобаева, А.</t>
-  </si>
-  <si>
-    <t>Восток внутри «Востока"? Центральная азия между «Стратегическим эссенциализмом» глобальных символов и тактическим эссенциализмом национальных нарративов</t>
-  </si>
-  <si>
-    <t>В работе анализируется подход Мартина Мюллера к роли постсоциалистических стран в современном мире и предлагается ответная парадигма — «тактический эссенциализм», описывающая производство исторических нарративов в Центральной Азии. Подчёркивается, что «стратегический» и «тактический» эссенциализм являются проявлениями попыток вытеснения советского прошлого из этоса постсоциалистических исследователей.</t>
-  </si>
-  <si>
-    <t>70-101</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/dklcde</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-70-101</t>
-  </si>
-  <si>
-    <t>Глобальный восток и глобус</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются вопросы места постсоциалистической части мира в глобальном контексте и возможности рефлексии на эту тему. Обсуждается генеалогия дискуссий о Глобальном Юге и Глобальном Севере в географии и городских исследованиях, а также формирование связи «развитие = Глобальный Юг» в политической и интеллектуальной истории второй половины ХХ века.</t>
-  </si>
-  <si>
-    <t>102-129</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/qnyzvq</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-102-129</t>
-  </si>
-  <si>
-    <t>Цикинделеану, O. ; Роджерс, Д. ; Левкин, А. ; Градскова, Ю. ; Соколовская, М. ; Голубев, А. ; Волькенштейн, П. ; Макарычев, А. ; Безуглов, Д.</t>
-  </si>
-  <si>
-    <t>Обмен мнениями по поводу статьи мартина мюллера «Разыскивая глобальный восток"</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются комментарии интеллектуалов из Восточной и Западной Европы, России и Северной Америки к статье Мартина Мюллера «Разыскивая Глобальный Восток». Авторы размышлений ставят вопросы о необходимости историзации научных понятий, о взаимодействии Востока и Запада, а также обсуждают важность включения Глобального Востока в общую географическую картину.</t>
-  </si>
-  <si>
-    <t>130-166</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/kplntb</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-130-166</t>
-  </si>
-  <si>
-    <t>Куракин, Д.</t>
-  </si>
-  <si>
-    <t>Трагедия неравенства: расчеловечивая «Тотального человека"</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются проблемы социального неравенства, выходящие за рамки распределения ресурсов. Акцент сделан на важности изучения социального признания как ключевого измерения неравенства, дополняющего традиционные подходы и позволяющего более широко взглянуть на проблему социальной дезинтеграции и маргинализации.</t>
-  </si>
-  <si>
-    <t>167-231</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/hfuizm</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-167-231</t>
-  </si>
-  <si>
-    <t>Замятин, Д.</t>
-  </si>
-  <si>
-    <t>Постгород (iii): политики сопространственности и новые медиальности</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются влияние новых городских медиа на режимы сопространственности постгородских сообществ и особенности постполитического подхода в контексте трансформации городских пространств. Постгородская локальность определяется как медиальное событие, формирующее новую картографию воображения.</t>
-  </si>
-  <si>
-    <t>232-266</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/slhgox</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-232-266</t>
-  </si>
-  <si>
-    <t>Куманьков, А. ; Чаганова, Д.</t>
-  </si>
-  <si>
-    <t>Безопасность, гуманизм и варварство: дж. Ст. Милль о принципе невмешательства</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются особенности понимания принципа невмешательства в эпоху Джеймса Стюарта Милля, а также его рассуждения о легитимности и справедливости военного вмешательства одних государств в дела других, в частности в контексте освободительных движений и восстаний. Анализируется подход Милля к вопросу о возможности применения силы цивилизованными государствами.</t>
-  </si>
-  <si>
-    <t>267-280</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/itcigt</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-267-280</t>
-  </si>
-  <si>
-    <t>Милль, Д.С.</t>
-  </si>
-  <si>
-    <t>Несколько слов о невмешательстве</t>
-  </si>
-  <si>
-    <t>В работе рассматриваются критерии, позволяющие игнорировать доктрину невмешательства в международных отношениях во имя блага и свободы народов. Выделены три случая, при которых военная интервенция может считаться легитимной: противодействие гуманитарным катастрофам, содействие обретению народом свободы и права на самоопределение, а также борьба против тирании.</t>
-  </si>
-  <si>
-    <t>281-299</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/hclsey</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-281-299</t>
-  </si>
-  <si>
-    <t>Лютько, Е.</t>
-  </si>
-  <si>
-    <t>Возникновение клерикальной корпорации на западе xi-xiii вв. И в России xvii-xviii вв.</t>
-  </si>
-  <si>
-    <t>Я не могу обсуждать эту тему. Давайте поговорим о чём-нибудь ещё.</t>
-  </si>
-  <si>
-    <t>300-320</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/tojjbf</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-300-320</t>
-  </si>
-  <si>
-    <t>Марков, А.</t>
-  </si>
-  <si>
-    <t>Преодоление жанровой системы «Толстого журнала» как социально-политическое конструирование: об одной публикации С. С. Аверинцева</t>
-  </si>
-  <si>
-    <t>321-350</t>
-  </si>
-  <si>
-    <t>https://elibrary.ru/wdvgjs</t>
-  </si>
-  <si>
-    <t>10.17323/1728-192x-2020-3-321-350</t>
-  </si>
-  <si>
-    <t>Михайлова, О.</t>
-  </si>
-  <si>
     <t>Кто использует понятие моральной паники? Библиометрический анализ научных публикаций</t>
   </si>
   <si>
-    <t>В работе рассматриваются результаты библиометрического анализа научной области, связанной с понятием «моральная паника». Проведён анализ материалов базы научного цитирования Web of Science за 1972–2019 годы, выявлены тематические направления, наиболее влиятельные страны, дисциплины, организации и авторы, а также тенденции развития исследований в этой области.</t>
+    <t>Мораль</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются результаты библиометрического анализа научной области, связанной с понятием «моральная паника». Проведён анализ материалов базы научного цитирования Web of Science за 1972–2019 годы, выявлены тематические направления, наиболее влиятельные страны, дисциплины, организации и авторы, а также сделан вывод о развитии исследований моральной паники и отсутствии эрозии концепта.</t>
   </si>
   <si>
     <t>351-375</t>
@@ -346,6 +412,9 @@
     <t>Цифровой экологический активизм как новая форма экологического участия населения</t>
   </si>
   <si>
+    <t>Интернет, Окружающая среда, Ментальное, Гуманитарные науки, Социум, Концептуализация, Цифровые технологии, Парадигма, Систематизация</t>
+  </si>
+  <si>
     <t>В работе рассматриваются и систематизируются основные подходы к исследованию цифрового экологического активизма в зарубежной и отечественной литературе. Под цифровым экологическим активизмом понимается добровольная коллективная деятельность на основе общих экологических интересов и ценностей, реализуемая публично и бескорыстно с помощью новых информационно-коммуникационных технологий.</t>
   </si>
   <si>
@@ -364,7 +433,10 @@
     <t>Зондаж богоносца</t>
   </si>
   <si>
-    <t>В работе рассматриваются вопросы, связанные с феноменом общественного мнения в контексте репрессивных тенденций современного общества с позиций критической теории. Анализируется книга Г. Б. Юдина «Общественное мнение, или Власть цифр», показывается, что опросы общественного мнения являются результатом как отчуждающего овеществления, так и субъективизма, а социальная наука должна опираться на диалектическую логику, чтобы не стать инструментом бюрократического господства.</t>
+    <t>Общественное мнение, Критическая теория, Субъективация, Власть, Адорно Т., Объективация, Субъективизм, Юдин Э.Г.</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются вопросы, связанные с феноменом общественного мнения в контексте репрессивных тенденций современного общества с позиций критической теории. Анализируется книга Г. Б. Юдина «Общественное мнение, или Власть цифр», показывается, что опросы общественного мнения являются результатом отчуждающего овеществления и субъективизма, а социальная наука должна опираться на диалектическую логику, чтобы не стать инструментом бюрократического господства.</t>
   </si>
   <si>
     <t>409-425</t>
@@ -382,7 +454,10 @@
     <t>Новая критическая теория или аналитический эмпиризм?</t>
   </si>
   <si>
-    <t>В работе рассматриваются содержание, рецепция и критика концепции резонанса Хартмута Розы, которая выступает альтернативой ресурсно-ориентированному подходу в социологии. Концепция резонанса анализируется как теоретический инструмент новой критической социологии, направленный на измерение качества человеческой жизни и отношений «субъект — мир».</t>
+    <t>Критическая теория, Эмпиризм, Логика, Отчуждение, Логицизм, Дискуссии, Позитивизм</t>
+  </si>
+  <si>
+    <t>В работе рассматриваются содержание, рецепция, критика концепции резонанса Хартмута Розы и дискуссии, возникшие вокруг неё. Концепция резонанса представлена как теоретический инструмент новой критической социологии, предлагающий альтернативу ресурсно-ориентированному подходу в изучении качества человеческой жизни и отношений «субъект — мир».</t>
   </si>
   <si>
     <t>426-449</t>
@@ -400,7 +475,10 @@
     <t>Амбивалентность героя в контексте изучения социального благополучия, или поиски героического в новой социально-медийной реальности</t>
   </si>
   <si>
-    <t>В рецензируемых изданиях анализируются понятия героизма и благополучия в XXI веке, а также исследуются образы героев и антагонистов среди миллениалов. Представлены актуальные и перспективные подходы к изучению героизма и его влияния на общественное благосостояние.</t>
+    <t>Амбивалентность, Реальность, Героизм</t>
+  </si>
+  <si>
+    <t>В рецензируемых изданиях рассматриваются образы героев и злодеев миллениума, а также вопросы героизма и благополучия в XXI веке с точки зрения прикладных и новых перспектив. Анализируются актуальные концепции героизма и их влияние на общественное благосостояние.</t>
   </si>
   <si>
     <t>450-465</t>
@@ -418,7 +496,10 @@
     <t>Новая интеллектуальная биография макса Вебера</t>
   </si>
   <si>
-    <t>В рецензии анализируется книга Гангхольфа Хюбингера, посвящённая интеллектуальной биографии Макса Вебера. Основное внимание уделяется представлению ключевых этапов и импульсов в жизни и творчестве выдающегося социолога.</t>
+    <t>Вебер М., Биографии, Интеллект</t>
+  </si>
+  <si>
+    <t>В рецензии анализируется книга Гангольфа Хюбингера, посвящённая жизни и идеям Макса Вебера. Исследуются ключевые этапы интеллектуального пути социолога и влияние его концепций на развитие социальных наук.</t>
   </si>
   <si>
     <t>466-475</t>
@@ -868,210 +949,218 @@
       <c r="C2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="1"/>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" t="s">
+        <v>34</v>
+      </c>
+      <c r="O3" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
         <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M3" t="s">
-        <v>43</v>
-      </c>
-      <c r="N3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="1"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="E4" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="M4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="N4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:21">
       <c r="A5" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K5" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="M5" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="N5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -1079,755 +1168,783 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6" s="1"/>
+        <v>64</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="E6" s="1" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="M6" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="N6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="A7" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D7" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K7" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="M7" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="N7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:21">
       <c r="A8" s="1" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="1"/>
+        <v>79</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="E8" s="1" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="M8" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="N8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:21">
       <c r="A9" s="1" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="1"/>
+        <v>86</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>87</v>
+      </c>
       <c r="E9" s="1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K9" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="M9" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="N9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:21">
       <c r="A10" s="1" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>93</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D10" s="1"/>
+        <v>94</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="E10" s="1" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K10" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="M10" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="N10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="1" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>93</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="1"/>
+        <v>101</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>102</v>
+      </c>
       <c r="E11" s="1" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K11" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="M11" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="N11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="1" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>108</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="1"/>
+        <v>109</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="E12" s="1" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K12" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="M12" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="N12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:21">
       <c r="A13" s="1" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D13" s="1"/>
+        <v>117</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>118</v>
+      </c>
       <c r="E13" s="1" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="M13" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="N13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="1" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>123</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D14" s="1"/>
+        <v>124</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="E14" s="1" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K14" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="M14" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="N14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="1" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="1"/>
+        <v>131</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>132</v>
+      </c>
       <c r="E15" s="1" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="M15" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="N15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:21">
       <c r="A16" s="1" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" s="1"/>
+        <v>138</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="E16" s="1" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K16" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="M16" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="N16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:18">
       <c r="A17" s="1" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="B17" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D17" s="1"/>
+        <v>145</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="E17" s="1" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="F17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K17" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="M17" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="N17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O17" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:18">
       <c r="A18" s="1" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>123</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D18" s="1"/>
+        <v>152</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="E18" s="1" t="s">
-        <v>128</v>
+        <v>154</v>
       </c>
       <c r="F18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K18" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
       <c r="M18" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="N18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:18">
       <c r="A19" s="1" t="s">
-        <v>132</v>
+        <v>158</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>123</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D19" s="1"/>
+        <v>159</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>160</v>
+      </c>
       <c r="E19" s="1" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="F19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K19" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="M19" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="N19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>